<commit_message>
docs: T:117 gait engine in protocol tables, READMEs, report correction
Instruction table (json+xlsx) gains the full T:117 entry with mode
table and the T:-117 completion event; state_table.yaml codebook adds
CRAWL_FWD/RUN_FWD (unverified until bench) and documents the takeover
rule; command counts 47->48. wavego_agent README documents the engine
fields and semantics (duration stays the supervisor's safety deadline;
turn-in-place falls back to T:111). Comparison report corrected: the
stock firmware was never lookup-table walking — closed-form IK with
analytic trajectories; the engine extends that, locomotion is still
not learned.
</commit_message>
<xml_diff>
--- a/wavego_pro_instruction_table.xlsx
+++ b/wavego_pro_instruction_table.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1172,127 +1172,135 @@
       <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>133</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CMD_PT_CTRL</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="A19" t="n">
+        <v>117</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CMD_GAIT_ENGINE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>body_motion</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Pan-tilt style body pose command (compat with UGV gimbal UI): maps X/Y onto body pitch/yaw posture.</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>X: float -180..180 -&gt; yaw -30..+30 deg; Y: float -30..30 -&gt; pitch -17.5..+17.5 deg</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>main.cpp -&gt; BodyCtrl::ptCtrl(X, Y) -&gt; pitchYawRoll(pitch, yaw, 0)</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>{"T": 133, "X": 0, "Y": 0}</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Parametric gait engine: mode (crawl/walk/run), continuous speed, body height, stride and distance targeting. All fields optional; speed&gt;0 starts/updates. Takeover commands (T:1/110/111/112/114/133) stop the engine.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>mode: int 0=crawl|1=walk|2=run; speed: float 0..1 (run capped 0.8 until verified); heading: float -180..180 (+left); height: float 75..110 mm; stride: float mm (0=mode default); distance: float mm (0=until stopped; &gt;0 auto-stop at target)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>main.cpp -&gt; BodyCtrl::configureEngine(...) -&gt; gait::Engine (GaitEngine.cpp)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>{"T": -117, "done": true, "traveled": mm, "cycles": n} (one-shot on distance completion)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>{"T": 117, "mode": 0, "speed": 0.5, "heading": 0, "height": 95, "stride": 0, "distance": 200}</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Modes: crawl duty 0.85 +CoM shift stride 12-30 delay 14-9ms; walk duty 0.75 stride 16-40 delay 8-4ms (stock); run duty 0.60 stride 32-24 delay 3-2ms. Distance integrates stride+2*acc per cycle.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>201</v>
+        <v>133</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>CMD_SET_COLOR</t>
+          <t>CMD_PT_CTRL</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>rgb_light</t>
+          <t>body_motion</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Set color of one RGB LED (2x WS2812/NeoPixel on GPIO26).</t>
+          <t>Pan-tilt style body pose command (compat with UGV gimbal UI): maps X/Y onto body pitch/yaw posture.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>set: int[4] = [id, r, g, b]; id: 0=left LED, 1=right LED; r/g/b: 0..255</t>
+          <t>X: float -180..180 -&gt; yaw -30..+30 deg; Y: float -30..30 -&gt; pitch -17.5..+17.5 deg</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; RGBLight::setColor(id, r, g, b) (Adafruit_NeoPixel, NEO_GRB + NEO_KHZ800)</t>
+          <t>main.cpp -&gt; BodyCtrl::ptCtrl(X, Y) -&gt; pitchYawRoll(pitch, yaw, 0)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>{"T": 201, "set": [0, 9, 0, 0]}</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Firmware quirk: RGBLight.cpp calls pixels.Color(g, r, b), so the red and green channels are swapped on the physical strip. Boot colors: LED0=(255,0,64), LED1=(64,0,255); assembly mode: both orange (255,64,0).</t>
-        </is>
-      </c>
+          <t>{"T": 133, "X": 0, "Y": 0}</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>CMD_DISPLAY_SINGLE</t>
+          <t>CMD_SET_COLOR</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>screen_oled</t>
+          <t>rgb_light</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Write one of the 4 text lines on the 128x32 SSD1306 OLED (I2C 0x3C).</t>
+          <t>Set color of one RGB LED (2x WS2812/NeoPixel on GPIO26).</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>line: int 1..4; text: string content of the line; update: bool 1=refresh panel now, 0=buffer only</t>
+          <t>set: int[4] = [id, r, g, b]; id: 0=left LED, 1=right LED; r/g/b: 0..255</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; ScreenCtrl::changeSingleLine(line, text, update)</t>
+          <t>main.cpp -&gt; RGBLight::setColor(id, r, g, b) (Adafruit_NeoPixel, NEO_GRB + NEO_KHZ800)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>{"T": 202, "line": 1, "text": "Hello, world!", "update": 1}</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr"/>
+          <t>{"T": 201, "set": [0, 9, 0, 0]}</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Firmware quirk: RGBLight.cpp calls pixels.Color(g, r, b), so the red and green channels are swapped on the physical strip. Boot colors: LED0=(255,0,64), LED1=(64,0,255); assembly mode: both orange (255,64,0).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CMD_DISPLAY_UPDATE</t>
+          <t>CMD_DISPLAY_SINGLE</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1302,34 +1310,34 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Refresh the OLED with the currently buffered 4 lines.</t>
+          <t>Write one of the 4 text lines on the 128x32 SSD1306 OLED (I2C 0x3C).</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>line: int 1..4; text: string content of the line; update: bool 1=refresh panel now, 0=buffer only</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; ScreenCtrl::updateFrame()</t>
+          <t>main.cpp -&gt; ScreenCtrl::changeSingleLine(line, text, update)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>{"T": 203}</t>
+          <t>{"T": 202, "line": 1, "text": "Hello, world!", "update": 1}</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>CMD_DISPLAY_FRAME</t>
+          <t>CMD_DISPLAY_UPDATE</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1339,38 +1347,34 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Write all 4 lines at once and refresh.</t>
+          <t>Refresh the OLED with the currently buffered 4 lines.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>l1: string line 1; l2: string line 2; l3: string line 3; l4: string line 4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; 4x changeSingleLine(...) with final update=true</t>
+          <t>main.cpp -&gt; ScreenCtrl::updateFrame()</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>{"T": 204, "l1": "Hello, world!", "l2": "Hello, world!", "l3": "Hello, world!", "l4": "Hello, world!"}</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>4 lines x 8px at text size 1; ~21 chars per line fit the 128px width.</t>
-        </is>
-      </c>
+          <t>{"T": 203}</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CMD_DISPLAY_CLEAR</t>
+          <t>CMD_DISPLAY_FRAME</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1380,122 +1384,122 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Clear the OLED.</t>
+          <t>Write all 4 lines at once and refresh.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>l1: string line 1; l2: string line 2; l3: string line 3; l4: string line 4</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; ScreenCtrl::clearDisplay()</t>
+          <t>main.cpp -&gt; 4x changeSingleLine(...) with final update=true</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>{"T": 205}</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
+          <t>{"T": 204, "l1": "Hello, world!", "l2": "Hello, world!", "l3": "Hello, world!", "l4": "Hello, world!"}</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>4 lines x 8px at text size 1; ~21 chars per line fit the 128px width.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>CMD_BUZZER_CTRL</t>
+          <t>CMD_DISPLAY_CLEAR</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>buzzer</t>
+          <t>screen_oled</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Active buzzer beep (GPIO21).</t>
+          <t>Clear the OLED.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>freq: int frequency in Hz; duration: int duration in ms (blocking)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; buzzerCtrl(freq, duration) (tone/noTone)</t>
+          <t>main.cpp -&gt; ScreenCtrl::clearDisplay()</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>{"T": 206, "freq": 1000, "duration": 10}</t>
+          <t>{"T": 205}</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>CMD_GET_BATTERY_VOLTAGE</t>
+          <t>CMD_BUZZER_CTRL</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>power</t>
+          <t>buzzer</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Read battery voltage via INA219 (I2C 0x42).</t>
+          <t>Active buzzer beep (GPIO21).</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>freq: int frequency in Hz; duration: int duration in ms (blocking)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; InaDataUpdate()</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>{"T": -207, "voltage": "float load voltage in V (2S 18650: ~6.4-8.4 V)"}</t>
-        </is>
-      </c>
+          <t>main.cpp -&gt; buzzerCtrl(freq, duration) (tone/noTone)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>{"T": 207}</t>
+          <t>{"T": 206, "freq": 1000, "duration": 10}</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>300</v>
+        <v>207</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>CMD_SCAN_FILES</t>
+          <t>CMD_GET_BATTERY_VOLTAGE</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>files_missions</t>
+          <t>power</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>List all mission files in LittleFS (printed to serial).</t>
+          <t>Read battery voltage via INA219 (I2C 0x42).</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1505,24 +1509,28 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::scan()</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
+          <t>main.cpp -&gt; InaDataUpdate()</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>{"T": -207, "voltage": "float load voltage in V (2S 18650: ~6.4-8.4 V)"}</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>{"T": 300}</t>
+          <t>{"T": 207}</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CMD_CREATE_MISSION</t>
+          <t>CMD_SCAN_FILES</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1532,34 +1540,34 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Create a mission file (/name.mission).</t>
+          <t>List all mission files in LittleFS (printed to serial).</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name; intro: string description comment</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::createMission(name, intro)</t>
+          <t>main.cpp -&gt; FilesCtrl::scan()</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>{"T": 301, "name": "mission1", "intro": "introduction for this mission file."}</t>
+          <t>{"T": 300}</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CMD_MISSION_CONTENT</t>
+          <t>CMD_CREATE_MISSION</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1569,34 +1577,34 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Print the content of a mission file (each step is one JSON command).</t>
+          <t>Create a mission file (/name.mission).</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name</t>
+          <t>name: string mission name; intro: string description comment</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::missionContent(name)</t>
+          <t>main.cpp -&gt; FilesCtrl::createMission(name, intro)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>{"T": 302, "name": "boot"}</t>
+          <t>{"T": 301, "name": "mission1", "intro": "introduction for this mission file."}</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CMD_APPEND_SETP_JSON</t>
+          <t>CMD_MISSION_CONTENT</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1606,34 +1614,34 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Append a JSON command as a new step at the end of a mission.</t>
+          <t>Print the content of a mission file (each step is one JSON command).</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name; json: string containing a full command JSON</t>
+          <t>name: string mission name</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::appendStep(name, json)</t>
+          <t>main.cpp -&gt; FilesCtrl::missionContent(name)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>{"T": 303, "name": "boot", "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
+          <t>{"T": 302, "name": "boot"}</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>CMD_INSERT_SETP_JSON</t>
+          <t>CMD_APPEND_SETP_JSON</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1643,34 +1651,34 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Insert a JSON command step before the given step number.</t>
+          <t>Append a JSON command as a new step at the end of a mission.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name; step: int step number (1-based); json: string command JSON</t>
+          <t>name: string mission name; json: string containing a full command JSON</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::insertStep(name, step, json)</t>
+          <t>main.cpp -&gt; FilesCtrl::appendStep(name, json)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>{"T": 304, "name": "boot", "step": 2, "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
+          <t>{"T": 303, "name": "boot", "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>CMD_REPLACE_SETP_JSON</t>
+          <t>CMD_INSERT_SETP_JSON</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1680,7 +1688,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Replace the JSON command at a given step number.</t>
+          <t>Insert a JSON command step before the given step number.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1690,24 +1698,24 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::replaceStep(name, step, json)</t>
+          <t>main.cpp -&gt; FilesCtrl::insertStep(name, step, json)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>{"T": 305, "name": "boot", "step": 2, "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
+          <t>{"T": 304, "name": "boot", "step": 2, "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CMD_DELETE_SETP</t>
+          <t>CMD_REPLACE_SETP_JSON</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1717,34 +1725,34 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Delete one step from a mission.</t>
+          <t>Replace the JSON command at a given step number.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name; step: int step number (1-based)</t>
+          <t>name: string mission name; step: int step number (1-based); json: string command JSON</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::deleteStep(name, step)</t>
+          <t>main.cpp -&gt; FilesCtrl::replaceStep(name, step, json)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>{"T": 306, "name": "boot", "step": 2}</t>
+          <t>{"T": 305, "name": "boot", "step": 2, "json": "{\"T\":201,\"set\":[0,9,0,0]}"}</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>CMD_RUN_STEP</t>
+          <t>CMD_DELETE_SETP</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1754,7 +1762,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Execute a single mission step immediately.</t>
+          <t>Delete one step from a mission.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1764,28 +1772,24 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; runStep(name, step) -&gt; jsonCmdReceiveHandler</t>
+          <t>main.cpp -&gt; FilesCtrl::deleteStep(name, step)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>{"T": 307, "name": "boot", "step": 2}</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Coupling function: the step itself is a full command JSON.</t>
-        </is>
-      </c>
+          <t>{"T": 306, "name": "boot", "step": 2}</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>CMD_RUN_MISSION</t>
+          <t>CMD_RUN_STEP</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1795,38 +1799,38 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Execute a whole mission, looping.</t>
+          <t>Execute a single mission step immediately.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name; interval: int ms delay between steps (50 ms internal time offset subtracted); loop: int loop count (-1 = infinite)</t>
+          <t>name: string mission name; step: int step number (1-based)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; runMission(name, interval, loop)</t>
+          <t>main.cpp -&gt; runStep(name, step) -&gt; jsonCmdReceiveHandler</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>{"T": 308, "name": "boot", "interval": 1000, "loop": 1}</t>
+          <t>{"T": 307, "name": "boot", "step": 2}</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Blocking; incoming serial data aborts the mission loop.</t>
+          <t>Coupling function: the step itself is a full command JSON.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>CMD_DELETE_MISSION</t>
+          <t>CMD_RUN_MISSION</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1836,34 +1840,38 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Delete a mission file.</t>
+          <t>Execute a whole mission, looping.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>name: string mission name</t>
+          <t>name: string mission name; interval: int ms delay between steps (50 ms internal time offset subtracted); loop: int loop count (-1 = infinite)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::deleteMission(name)</t>
+          <t>main.cpp -&gt; runMission(name, interval, loop)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>{"T": 309, "name": "boot"}</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr"/>
+          <t>{"T": 308, "name": "boot", "interval": 1000, "loop": 1}</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Blocking; incoming serial data aborts the mission loop.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>399</v>
+        <v>309</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>CMD_FORMAT_FLASH</t>
+          <t>CMD_DELETE_MISSION</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1873,75 +1881,71 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Format LittleFS (wipes ALL missions, including 'boot' WiFi/calibration config).</t>
+          <t>Delete a mission file.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>name: string mission name</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::flash() -&gt; LittleFS.format()</t>
+          <t>main.cpp -&gt; FilesCtrl::deleteMission(name)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>{"T": 399}</t>
+          <t>{"T": 309, "name": "boot"}</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>CMD_SET_WIFI_MODE</t>
+          <t>CMD_FORMAT_FLASH</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>wireless_wifi</t>
+          <t>files_missions</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Configure WiFi AP and/or STA credentials; result is persisted into the 'boot' mission (auto-applied at power-on).</t>
+          <t>Format LittleFS (wipes ALL missions, including 'boot' WiFi/calibration config).</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>mode: int 0 = clear/reset wifi config, 1 = set AP(+STA) config; ap_ssid: string AP SSID; ap_password: string AP password (min 8 chars); channel: int WiFi channel; sta_ssid: string STA SSID (empty = AP only); sta_password: string STA password</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::setWifiMode(...) + FilesCtrl::checkReplaceStep('boot', echo)</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Echo of the stored config as {"T":400,...}</t>
-        </is>
-      </c>
+          <t>main.cpp -&gt; FilesCtrl::flash() -&gt; LittleFS.format()</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>{"T": 400, "mode": 1, "ap_ssid": "WAVEGO", "ap_password": "12345678", "channel": 1, "sta_ssid": "", "sta_password": ""}</t>
+          <t>{"T": 399}</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>CMD_WIFI_INFO</t>
+          <t>CMD_SET_WIFI_MODE</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1951,34 +1955,38 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Print the stored WiFi config command from the 'boot' mission.</t>
+          <t>Configure WiFi AP and/or STA credentials; result is persisted into the 'boot' mission (auto-applied at power-on).</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mode: int 0 = clear/reset wifi config, 1 = set AP(+STA) config; ap_ssid: string AP SSID; ap_password: string AP password (min 8 chars); channel: int WiFi channel; sta_ssid: string STA SSID (empty = AP only); sta_password: string STA password</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; FilesCtrl::findCmdByType('boot', CMD_SET_WIFI_MODE)</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
+          <t>main.cpp -&gt; Wireless::setWifiMode(...) + FilesCtrl::checkReplaceStep('boot', echo)</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Echo of the stored config as {"T":400,...}</t>
+        </is>
+      </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>{"T": 401}</t>
+          <t>{"T": 400, "mode": 1, "ap_ssid": "WAVEGO", "ap_password": "12345678", "channel": 1, "sta_ssid": "", "sta_password": ""}</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CMD_GET_AP_IP</t>
+          <t>CMD_WIFI_INFO</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1988,7 +1996,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Print the AP-mode IP address.</t>
+          <t>Print the stored WiFi config command from the 'boot' mission.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1998,24 +2006,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::getAPIP()</t>
+          <t>main.cpp -&gt; FilesCtrl::findCmdByType('boot', CMD_SET_WIFI_MODE)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>{"T": 402}</t>
+          <t>{"T": 401}</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>CMD_GET_STA_IP</t>
+          <t>CMD_GET_AP_IP</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2025,7 +2033,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Print the STA-mode IP address.</t>
+          <t>Print the AP-mode IP address.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2035,61 +2043,61 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::getSTAIP()</t>
+          <t>main.cpp -&gt; Wireless::getAPIP()</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>{"T": 403}</t>
+          <t>{"T": 402}</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>CMD_INIT_ESP_NOW</t>
+          <t>CMD_GET_STA_IP</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>esp_now</t>
+          <t>wireless_wifi</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Initialize ESP-NOW.</t>
+          <t>Print the STA-mode IP address.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>longrange: bool enable long-range mode</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::espnowInit(longrange)</t>
+          <t>main.cpp -&gt; Wireless::getSTAIP()</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>{"T": 410, "longrange": 0}</t>
+          <t>{"T": 403}</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>CMD_SET_ESP_NOW_MODE</t>
+          <t>CMD_INIT_ESP_NOW</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2099,34 +2107,34 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Enable/disable ESP-NOW receive.</t>
+          <t>Initialize ESP-NOW.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>mode: int 0 = off, 1 = on (default)</t>
+          <t>longrange: bool enable long-range mode</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::setEspNowMode(mode)</t>
+          <t>main.cpp -&gt; Wireless::espnowInit(longrange)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>{"T": 411, "mode": 1}</t>
+          <t>{"T": 410, "longrange": 0}</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>CMD_GET_MAC</t>
+          <t>CMD_SET_ESP_NOW_MODE</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2136,34 +2144,34 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Print this device's MAC address.</t>
+          <t>Enable/disable ESP-NOW receive.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mode: int 0 = off, 1 = on (default)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::macToString(Wireless::getMac())</t>
+          <t>main.cpp -&gt; Wireless::setEspNowMode(mode)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>{"T": 412}</t>
+          <t>{"T": 411, "mode": 1}</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>CMD_ESP_NOW_SEND</t>
+          <t>CMD_GET_MAC</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2173,34 +2181,34 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Send a JSON payload to a peer over ESP-NOW.</t>
+          <t>Print this device's MAC address.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>mac: string peer MAC ('FF,FF,FF,FF,FF,FF' format); data: string JSON command to deliver</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::sendEspNow(mac, data)</t>
+          <t>main.cpp -&gt; Wireless::macToString(Wireless::getMac())</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>{"T": 413, "mac": "FF,FF,FF,FF,FF,FF", "data": "{\"T\":205,\"freq\":500,\"duration\":30}"}</t>
+          <t>{"T": 412}</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>CMD_ADD_MAC</t>
+          <t>CMD_ESP_NOW_SEND</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2210,71 +2218,71 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Register a peer MAC for ESP-NOW broadcast.</t>
+          <t>Send a JSON payload to a peer over ESP-NOW.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>mac: string peer MAC ('FF:FF:FF:FF:FF:FF' format)</t>
+          <t>mac: string peer MAC ('FF,FF,FF,FF,FF,FF' format); data: string JSON command to deliver</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; Wireless::addMacToPeerString(mac)</t>
+          <t>main.cpp -&gt; Wireless::sendEspNow(mac, data)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>{"T": 414, "mac": "FF:FF:FF:FF:FF:FF"}</t>
+          <t>{"T": 413, "mac": "FF,FF,FF,FF,FF,FF", "data": "{\"T\":205,\"freq\":500,\"duration\":30}"}</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>600</v>
+        <v>414</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>ESP32_REBOOT</t>
+          <t>CMD_ADD_MAC</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>esp_now</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Reboot the ESP32.</t>
+          <t>Register a peer MAC for ESP-NOW broadcast.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mac: string peer MAC ('FF:FF:FF:FF:FF:FF' format)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; ESP.restart()</t>
+          <t>main.cpp -&gt; Wireless::addMacToPeerString(mac)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>{"T": 600}</t>
+          <t>{"T": 414, "mac": "FF:FF:FF:FF:FF:FF"}</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>CMD_CLEAR_NVS</t>
+          <t>ESP32_REBOOT</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2284,7 +2292,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Erase and re-init NVS flash.</t>
+          <t>Reboot the ESP32.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2294,16 +2302,53 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>main.cpp -&gt; nvs_flash_erase() + nvs_flash_init()</t>
+          <t>main.cpp -&gt; ESP.restart()</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
+          <t>{"T": 600}</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>601</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>CMD_CLEAR_NVS</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Erase and re-init NVS flash.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>main.cpp -&gt; nvs_flash_erase() + nvs_flash_init()</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
           <t>{"T": 601}</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I48"/>

</xml_diff>